<commit_message>
Regenerate benchmark Excel with streaming TTFP (STT) + network-removed latency (TTS)
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/benchmark/Voice_Benchmark.xlsx
+++ b/benchmark/Voice_Benchmark.xlsx
@@ -469,7 +469,7 @@
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>A fair side-by-side test. The SAME text (for speech) and the SAME audio (for transcription) were sent to every provider, and the real results were measured. No numbers are estimated or made up — everything was measured live from the APIs.</t>
+          <t>A fair side-by-side test. The SAME text (speech) and the SAME audio (transcription) were sent to each provider and the real results measured. No numbers are invented.</t>
         </is>
       </c>
     </row>
@@ -481,49 +481,57 @@
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>2026-10-29 10:59:13</t>
+          <t>2026-10-29 11:49:41</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="2" t="inlineStr"/>
-      <c r="B6" s="3" t="inlineStr"/>
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>TTS compared</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="inlineStr">
+        <is>
+          <t>Atlas (atlas-speak), ElevenLabs, Cartesia, Deepgram (Aura, English only).</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="4" t="inlineStr">
         <is>
-          <t>TTS = Text To Speech</t>
+          <t>STT compared</t>
         </is>
       </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
-          <t>Turning written text into spoken audio. Compared: Atlas (atlas-speak), ElevenLabs, Cartesia.</t>
+          <t>Atlas (atlas-listen), ElevenLabs (Scribe), Deepgram, AssemblyAI.</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="4" t="inlineStr">
-        <is>
-          <t>STT = Speech To Text</t>
-        </is>
-      </c>
-      <c r="B8" s="3" t="inlineStr">
-        <is>
-          <t>Turning spoken audio into written text. Compared: Atlas (atlas-listen), Deepgram, AssemblyAI.</t>
-        </is>
-      </c>
+      <c r="A8" s="2" t="inlineStr"/>
+      <c r="B8" s="3" t="inlineStr"/>
     </row>
     <row r="9">
-      <c r="A9" s="2" t="inlineStr"/>
+      <c r="A9" s="1" t="inlineStr">
+        <is>
+          <t>--- TTS parameters (plain English) ---</t>
+        </is>
+      </c>
       <c r="B9" s="3" t="inlineStr"/>
     </row>
     <row r="10">
-      <c r="A10" s="1" t="inlineStr">
-        <is>
-          <t>--- TTS parameters (plain English) ---</t>
-        </is>
-      </c>
-      <c r="B10" s="3" t="inlineStr"/>
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>Processing latency (ms)</t>
+        </is>
+      </c>
+      <c r="B10" s="3" t="inlineStr">
+        <is>
+          <t>The MAIN number. Time until the first audio comes out, with the NETWORK REMOVED (we measure the round-trip to each provider and subtract it). This shows the provider's OWN speed, not where we run from. Lower = better.</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="4" t="inlineStr">
@@ -533,57 +541,57 @@
       </c>
       <c r="B11" s="3" t="inlineStr">
         <is>
-          <t>How long until the FIRST piece of audio comes back after we send the text. Lower = the voice starts sooner = feels faster. Measured on our machine over the real internet, so it includes network time.</t>
+          <t>Time until the first audio byte reaches us, INCLUDING the network. Shown for transparency; processing = first-byte minus network round-trip.</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="4" t="inlineStr">
         <is>
-          <t>First-byte median</t>
+          <t>Total time (ms)</t>
         </is>
       </c>
       <c r="B12" s="3" t="inlineStr">
         <is>
-          <t>The middle value across repeated runs (we ran each sentence 3 times). Median is used so one slow run doesn't skew it.</t>
+          <t>Time until the whole audio clip is received.</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="4" t="inlineStr">
         <is>
-          <t>Total time (ms)</t>
+          <t>Median</t>
         </is>
       </c>
       <c r="B13" s="3" t="inlineStr">
         <is>
-          <t>How long until the WHOLE audio clip is received.</t>
+          <t>Middle value across 3 runs per sentence (so one slow run doesn't skew it).</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="4" t="inlineStr">
-        <is>
-          <t>Provider-reported first audio (ms)</t>
-        </is>
-      </c>
-      <c r="B14" s="3" t="inlineStr">
-        <is>
-          <t>Atlas also reports its OWN internal time-to-first-audio in a header. This is Atlas's number measured inside Atlas (no network). Other providers do not report this, so it is blank for them.</t>
-        </is>
-      </c>
+      <c r="A14" s="2" t="inlineStr"/>
+      <c r="B14" s="3" t="inlineStr"/>
     </row>
     <row r="15">
-      <c r="A15" s="2" t="inlineStr"/>
+      <c r="A15" s="1" t="inlineStr">
+        <is>
+          <t>--- STT parameters (plain English) ---</t>
+        </is>
+      </c>
       <c r="B15" s="3" t="inlineStr"/>
     </row>
     <row r="16">
-      <c r="A16" s="1" t="inlineStr">
-        <is>
-          <t>--- STT parameters (plain English) ---</t>
-        </is>
-      </c>
-      <c r="B16" s="3" t="inlineStr"/>
+      <c r="A16" s="4" t="inlineStr">
+        <is>
+          <t>Latency (ms)</t>
+        </is>
+      </c>
+      <c r="B16" s="3" t="inlineStr">
+        <is>
+          <t>For Atlas and Deepgram: STREAMING 'time to first word' — audio is streamed to their realtime API and we time the first word (the metric that matters for a live voice agent, same as the speech-to-speech model). For AssemblyAI and ElevenLabs: batch mode, so compare their ACCURACY, not their latency.</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="4" t="inlineStr">
@@ -605,7 +613,7 @@
       </c>
       <c r="B18" s="3" t="inlineStr">
         <is>
-          <t>Word Error Rate — the share of WORDS that were wrong. Accuracy = 100% minus WER.</t>
+          <t>Word Error Rate — share of WORDS wrong. Accuracy = 100% minus WER.</t>
         </is>
       </c>
     </row>
@@ -617,91 +625,91 @@
       </c>
       <c r="B19" s="3" t="inlineStr">
         <is>
-          <t>Character Error Rate — the share of CHARACTERS that were wrong. Used for Japanese because Japanese has no spaces between words, so characters are the fair unit.</t>
+          <t>Character Error Rate — share of CHARACTERS wrong. Used for Japanese (no spaces between words).</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="4" t="inlineStr">
         <is>
-          <t>Latency (ms)</t>
+          <t>Mode</t>
         </is>
       </c>
       <c r="B20" s="3" t="inlineStr">
         <is>
-          <t>How long the provider took to return the transcript.</t>
+          <t>'streaming (time to first word)' = realtime. 'batch' = whole file processed at once.</t>
         </is>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="4" t="inlineStr">
-        <is>
-          <t>Mode</t>
-        </is>
-      </c>
-      <c r="B21" s="3" t="inlineStr">
-        <is>
-          <t>'sync' = answers in one request (real-time style). 'batch (upload+poll)' = AssemblyAI uploads the file then we wait for it, so its latency is NOT comparable to real-time STT — compare its ACCURACY.</t>
-        </is>
-      </c>
+      <c r="A21" s="2" t="inlineStr"/>
+      <c r="B21" s="3" t="inlineStr"/>
     </row>
     <row r="22">
-      <c r="A22" s="2" t="inlineStr"/>
+      <c r="A22" s="1" t="inlineStr">
+        <is>
+          <t>--- Honest notes ---</t>
+        </is>
+      </c>
       <c r="B22" s="3" t="inlineStr"/>
     </row>
     <row r="23">
-      <c r="A23" s="1" t="inlineStr">
-        <is>
-          <t>--- Honest notes / caveats ---</t>
-        </is>
-      </c>
-      <c r="B23" s="3" t="inlineStr"/>
+      <c r="A23" s="4" t="inlineStr">
+        <is>
+          <t>Fairness</t>
+        </is>
+      </c>
+      <c r="B23" s="3" t="inlineStr">
+        <is>
+          <t>All measured the same way, at the same time, from one machine. The relative comparison is the point.</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="4" t="inlineStr">
         <is>
-          <t>Where it ran</t>
+          <t>STT test audio</t>
         </is>
       </c>
       <c r="B24" s="3" t="inlineStr">
         <is>
-          <t>All tests ran from one machine over normal internet. Absolute latency depends on network distance to each provider's servers. The FAIR takeaway is the RELATIVE comparison between providers, measured the same way at the same time.</t>
+          <t>Clean speech generated by a TTS voice (ElevenLabs); the SAME clip is sent to every STT provider. Real noisy phone calls may score differently.</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="4" t="inlineStr">
         <is>
-          <t>STT test audio</t>
+          <t>Number formatting</t>
         </is>
       </c>
       <c r="B25" s="3" t="inlineStr">
         <is>
-          <t>The audio used for the transcription test was generated by a text-to-speech voice (ElevenLabs), so it is clean studio-like speech. Real phone calls with noise/accents may score differently. It is the SAME clip for every STT provider, so the comparison is fair.</t>
+          <t>Sentences with numbers (e.g. 'five thousand dollars') lower accuracy for everyone because engines format them differently ('$5,000'); it's an equal penalty, not a real error.</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="4" t="inlineStr">
         <is>
-          <t>Voices used</t>
+          <t>Deepgram TTS</t>
         </is>
       </c>
       <c r="B26" s="3" t="inlineStr">
         <is>
-          <t>Each TTS provider used an appropriate voice for the language. Atlas's voices are Japanese, so its English is spoken with a Japanese voice.</t>
+          <t>English only (Aura). Japanese shows N/A.</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="4" t="inlineStr">
         <is>
-          <t>Pricing</t>
+          <t>ElevenLabs STT</t>
         </is>
       </c>
       <c r="B27" s="3" t="inlineStr">
         <is>
-          <t>Not measured here. Check each provider's pricing page; it changes often.</t>
+          <t>Needs the Speech-to-Text permission on the key; 0% means the permission is off.</t>
         </is>
       </c>
     </row>
@@ -716,17 +724,15 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H7"/>
+  <dimension ref="A1:F9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="13" customWidth="1" min="1" max="1"/>
-    <col width="10" customWidth="1" min="2" max="2"/>
-    <col width="28" customWidth="1" min="3" max="3"/>
-    <col width="20" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="9" customWidth="1" min="2" max="2"/>
+    <col width="42" customWidth="1" min="3" max="3"/>
+    <col width="38" customWidth="1" min="4" max="4"/>
     <col width="20" customWidth="1" min="5" max="5"/>
-    <col width="22" customWidth="1" min="6" max="6"/>
-    <col width="30" customWidth="1" min="7" max="7"/>
-    <col width="12" customWidth="1" min="8" max="8"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -742,30 +748,20 @@
       </c>
       <c r="C1" s="5" t="inlineStr">
         <is>
-          <t>First-byte latency — median (ms)</t>
+          <t>Processing latency — median (ms) [network removed]</t>
         </is>
       </c>
       <c r="D1" s="5" t="inlineStr">
         <is>
-          <t>First-byte — best (ms)</t>
+          <t>First-byte — median (ms) [incl. network]</t>
         </is>
       </c>
       <c r="E1" s="5" t="inlineStr">
         <is>
-          <t>First-byte — worst (ms)</t>
+          <t>Total — median (ms)</t>
         </is>
       </c>
       <c r="F1" s="5" t="inlineStr">
-        <is>
-          <t>Total time — median (ms)</t>
-        </is>
-      </c>
-      <c r="G1" s="5" t="inlineStr">
-        <is>
-          <t>Atlas's own reported first-audio (ms)</t>
-        </is>
-      </c>
-      <c r="H1" s="5" t="inlineStr">
         <is>
           <t>Sentences OK</t>
         </is>
@@ -783,21 +779,15 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>977</v>
+        <v>1298</v>
       </c>
       <c r="D2" t="n">
-        <v>936</v>
+        <v>1408</v>
       </c>
       <c r="E2" t="n">
-        <v>1146</v>
-      </c>
-      <c r="F2" t="n">
-        <v>2564</v>
-      </c>
-      <c r="G2" t="n">
-        <v>403</v>
-      </c>
-      <c r="H2" t="inlineStr">
+        <v>2836</v>
+      </c>
+      <c r="F2" t="inlineStr">
         <is>
           <t>4/4</t>
         </is>
@@ -815,21 +805,15 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>953</v>
+        <v>1006</v>
       </c>
       <c r="D3" t="n">
-        <v>919</v>
+        <v>1117</v>
       </c>
       <c r="E3" t="n">
-        <v>989</v>
-      </c>
-      <c r="F3" t="n">
-        <v>2134</v>
-      </c>
-      <c r="G3" t="n">
-        <v>334</v>
-      </c>
-      <c r="H3" t="inlineStr">
+        <v>2427</v>
+      </c>
+      <c r="F3" t="inlineStr">
         <is>
           <t>4/4</t>
         </is>
@@ -847,19 +831,15 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>437</v>
+        <v>625</v>
       </c>
       <c r="D4" t="n">
-        <v>400</v>
+        <v>629</v>
       </c>
       <c r="E4" t="n">
-        <v>466</v>
-      </c>
-      <c r="F4" t="n">
-        <v>1011</v>
-      </c>
-      <c r="G4" t="inlineStr"/>
-      <c r="H4" t="inlineStr">
+        <v>1226</v>
+      </c>
+      <c r="F4" t="inlineStr">
         <is>
           <t>4/4</t>
         </is>
@@ -877,19 +857,15 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>420</v>
+        <v>676</v>
       </c>
       <c r="D5" t="n">
-        <v>399</v>
+        <v>680</v>
       </c>
       <c r="E5" t="n">
-        <v>427</v>
-      </c>
-      <c r="F5" t="n">
-        <v>1086</v>
-      </c>
-      <c r="G5" t="inlineStr"/>
-      <c r="H5" t="inlineStr">
+        <v>1274</v>
+      </c>
+      <c r="F5" t="inlineStr">
         <is>
           <t>4/4</t>
         </is>
@@ -898,7 +874,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>ElevenLabs</t>
+          <t>Deepgram</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -907,19 +883,15 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>683</v>
+        <v>1051</v>
       </c>
       <c r="D6" t="n">
-        <v>595</v>
+        <v>1290</v>
       </c>
       <c r="E6" t="n">
-        <v>693</v>
-      </c>
-      <c r="F6" t="n">
-        <v>801</v>
-      </c>
-      <c r="G6" t="inlineStr"/>
-      <c r="H6" t="inlineStr">
+        <v>1524</v>
+      </c>
+      <c r="F6" t="inlineStr">
         <is>
           <t>4/4</t>
         </is>
@@ -928,28 +900,82 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
+          <t>Deepgram</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>0/4</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
           <t>ElevenLabs</t>
         </is>
       </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>ja</t>
-        </is>
-      </c>
-      <c r="C7" t="n">
-        <v>678</v>
-      </c>
-      <c r="D7" t="n">
-        <v>647</v>
-      </c>
-      <c r="E7" t="n">
-        <v>702</v>
-      </c>
-      <c r="F7" t="n">
-        <v>772</v>
-      </c>
-      <c r="G7" t="inlineStr"/>
-      <c r="H7" t="inlineStr">
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>en</t>
+        </is>
+      </c>
+      <c r="C8" t="n">
+        <v>740</v>
+      </c>
+      <c r="D8" t="n">
+        <v>766</v>
+      </c>
+      <c r="E8" t="n">
+        <v>891</v>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>4/4</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>ElevenLabs</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="C9" t="n">
+        <v>824</v>
+      </c>
+      <c r="D9" t="n">
+        <v>856</v>
+      </c>
+      <c r="E9" t="n">
+        <v>940</v>
+      </c>
+      <c r="F9" t="inlineStr">
         <is>
           <t>4/4</t>
         </is>
@@ -966,16 +992,15 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G7"/>
+  <dimension ref="A1:F9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="13" customWidth="1" min="1" max="1"/>
-    <col width="10" customWidth="1" min="2" max="2"/>
-    <col width="9" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="9" customWidth="1" min="2" max="2"/>
+    <col width="8" customWidth="1" min="3" max="3"/>
     <col width="20" customWidth="1" min="4" max="4"/>
     <col width="20" customWidth="1" min="5" max="5"/>
-    <col width="22" customWidth="1" min="6" max="6"/>
-    <col width="11" customWidth="1" min="7" max="7"/>
+    <col width="34" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1009,11 +1034,6 @@
           <t>Mode</t>
         </is>
       </c>
-      <c r="G1" s="5" t="inlineStr">
-        <is>
-          <t>Sentences</t>
-        </is>
-      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -1035,15 +1055,12 @@
         <v>83.8</v>
       </c>
       <c r="E2" t="n">
-        <v>5764</v>
+        <v>5890</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
           <t>batch (upload+poll)</t>
         </is>
-      </c>
-      <c r="G2" t="n">
-        <v>4</v>
       </c>
     </row>
     <row r="3">
@@ -1063,18 +1080,15 @@
         </is>
       </c>
       <c r="D3" t="n">
-        <v>97</v>
+        <v>99.2</v>
       </c>
       <c r="E3" t="n">
-        <v>5172</v>
+        <v>6259</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
           <t>batch (upload+poll)</t>
         </is>
-      </c>
-      <c r="G3" t="n">
-        <v>4</v>
       </c>
     </row>
     <row r="4">
@@ -1097,15 +1111,12 @@
         <v>83.8</v>
       </c>
       <c r="E4" t="n">
-        <v>2606</v>
+        <v>374</v>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>sync</t>
-        </is>
-      </c>
-      <c r="G4" t="n">
-        <v>4</v>
+          <t>streaming (time to first word)</t>
+        </is>
       </c>
     </row>
     <row r="5">
@@ -1125,18 +1136,15 @@
         </is>
       </c>
       <c r="D5" t="n">
-        <v>98.90000000000001</v>
+        <v>100</v>
       </c>
       <c r="E5" t="n">
-        <v>2531</v>
+        <v>451</v>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>sync</t>
-        </is>
-      </c>
-      <c r="G5" t="n">
-        <v>4</v>
+          <t>streaming (time to first word)</t>
+        </is>
       </c>
     </row>
     <row r="6">
@@ -1156,18 +1164,15 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>83.8</v>
+        <v>100</v>
       </c>
       <c r="E6" t="n">
-        <v>1390</v>
+        <v>732</v>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>sync</t>
-        </is>
-      </c>
-      <c r="G6" t="n">
-        <v>4</v>
+          <t>streaming (time to first word)</t>
+        </is>
       </c>
     </row>
     <row r="7">
@@ -1187,18 +1192,71 @@
         </is>
       </c>
       <c r="D7" t="n">
-        <v>100</v>
+        <v>99.2</v>
       </c>
       <c r="E7" t="n">
-        <v>2039</v>
+        <v>772</v>
       </c>
       <c r="F7" t="inlineStr">
         <is>
+          <t>streaming (time to first word)</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>ElevenLabs</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>en</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>WER</t>
+        </is>
+      </c>
+      <c r="D8" t="n">
+        <v>0</v>
+      </c>
+      <c r="E8" t="n">
+        <v>1144</v>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
           <t>sync</t>
         </is>
       </c>
-      <c r="G7" t="n">
-        <v>4</v>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>ElevenLabs</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>CER</t>
+        </is>
+      </c>
+      <c r="D9" t="n">
+        <v>0</v>
+      </c>
+      <c r="E9" t="n">
+        <v>1550</v>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>sync</t>
+        </is>
       </c>
     </row>
   </sheetData>
@@ -1212,20 +1270,18 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K25"/>
+  <dimension ref="A1:I33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
     <col width="9" customWidth="1" min="2" max="2"/>
     <col width="4" customWidth="1" min="3" max="3"/>
     <col width="55" customWidth="1" min="4" max="4"/>
-    <col width="20" customWidth="1" min="5" max="5"/>
-    <col width="8" customWidth="1" min="6" max="6"/>
-    <col width="8" customWidth="1" min="7" max="7"/>
-    <col width="18" customWidth="1" min="8" max="8"/>
-    <col width="28" customWidth="1" min="9" max="9"/>
-    <col width="9" customWidth="1" min="10" max="10"/>
-    <col width="9" customWidth="1" min="11" max="11"/>
+    <col width="16" customWidth="1" min="5" max="5"/>
+    <col width="16" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
+    <col width="9" customWidth="1" min="8" max="8"/>
+    <col width="16" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1251,35 +1307,25 @@
       </c>
       <c r="E1" s="5" t="inlineStr">
         <is>
-          <t>First-byte median (ms)</t>
+          <t>Processing (ms)</t>
         </is>
       </c>
       <c r="F1" s="5" t="inlineStr">
         <is>
-          <t>best</t>
+          <t>First-byte (ms)</t>
         </is>
       </c>
       <c r="G1" s="5" t="inlineStr">
         <is>
-          <t>worst</t>
+          <t>Total (ms)</t>
         </is>
       </c>
       <c r="H1" s="5" t="inlineStr">
         <is>
-          <t>Total median (ms)</t>
+          <t>Runs OK</t>
         </is>
       </c>
       <c r="I1" s="5" t="inlineStr">
-        <is>
-          <t>Atlas reported first-audio (ms)</t>
-        </is>
-      </c>
-      <c r="J1" s="5" t="inlineStr">
-        <is>
-          <t>Runs OK</t>
-        </is>
-      </c>
-      <c r="K1" s="5" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
@@ -1305,26 +1351,20 @@
         </is>
       </c>
       <c r="E2" t="n">
-        <v>936</v>
+        <v>1263</v>
       </c>
       <c r="F2" t="n">
-        <v>909</v>
+        <v>1375</v>
       </c>
       <c r="G2" t="n">
-        <v>945</v>
-      </c>
-      <c r="H2" t="n">
-        <v>2279</v>
+        <v>2787</v>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>3/3</t>
+        </is>
       </c>
       <c r="I2" t="n">
-        <v>347</v>
-      </c>
-      <c r="J2" t="inlineStr">
-        <is>
-          <t>3/3</t>
-        </is>
-      </c>
-      <c r="K2" t="n">
         <v>200</v>
       </c>
     </row>
@@ -1348,26 +1388,20 @@
         </is>
       </c>
       <c r="E3" t="n">
-        <v>1146</v>
+        <v>1334</v>
       </c>
       <c r="F3" t="n">
-        <v>920</v>
+        <v>1442</v>
       </c>
       <c r="G3" t="n">
-        <v>1217</v>
-      </c>
-      <c r="H3" t="n">
-        <v>2803</v>
+        <v>2757</v>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>3/3</t>
+        </is>
       </c>
       <c r="I3" t="n">
-        <v>650</v>
-      </c>
-      <c r="J3" t="inlineStr">
-        <is>
-          <t>3/3</t>
-        </is>
-      </c>
-      <c r="K3" t="n">
         <v>200</v>
       </c>
     </row>
@@ -1391,26 +1425,20 @@
         </is>
       </c>
       <c r="E4" t="n">
-        <v>971</v>
+        <v>1394</v>
       </c>
       <c r="F4" t="n">
-        <v>908</v>
+        <v>1501</v>
       </c>
       <c r="G4" t="n">
-        <v>987</v>
-      </c>
-      <c r="H4" t="n">
-        <v>2326</v>
+        <v>2885</v>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>3/3</t>
+        </is>
       </c>
       <c r="I4" t="n">
-        <v>420</v>
-      </c>
-      <c r="J4" t="inlineStr">
-        <is>
-          <t>3/3</t>
-        </is>
-      </c>
-      <c r="K4" t="n">
         <v>200</v>
       </c>
     </row>
@@ -1434,26 +1462,20 @@
         </is>
       </c>
       <c r="E5" t="n">
-        <v>983</v>
+        <v>1169</v>
       </c>
       <c r="F5" t="n">
-        <v>961</v>
+        <v>1276</v>
       </c>
       <c r="G5" t="n">
-        <v>1144</v>
-      </c>
-      <c r="H5" t="n">
-        <v>3148</v>
+        <v>3229</v>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>3/3</t>
+        </is>
       </c>
       <c r="I5" t="n">
-        <v>387</v>
-      </c>
-      <c r="J5" t="inlineStr">
-        <is>
-          <t>3/3</t>
-        </is>
-      </c>
-      <c r="K5" t="n">
         <v>200</v>
       </c>
     </row>
@@ -1477,23 +1499,20 @@
         </is>
       </c>
       <c r="E6" t="n">
-        <v>595</v>
+        <v>858</v>
       </c>
       <c r="F6" t="n">
-        <v>590</v>
+        <v>885</v>
       </c>
       <c r="G6" t="n">
-        <v>622</v>
-      </c>
-      <c r="H6" t="n">
-        <v>728</v>
-      </c>
-      <c r="J6" t="inlineStr">
+        <v>1016</v>
+      </c>
+      <c r="H6" t="inlineStr">
         <is>
           <t>3/3</t>
         </is>
       </c>
-      <c r="K6" t="n">
+      <c r="I6" t="n">
         <v>200</v>
       </c>
     </row>
@@ -1517,23 +1536,20 @@
         </is>
       </c>
       <c r="E7" t="n">
-        <v>677</v>
+        <v>845</v>
       </c>
       <c r="F7" t="n">
-        <v>560</v>
+        <v>872</v>
       </c>
       <c r="G7" t="n">
-        <v>694</v>
-      </c>
-      <c r="H7" t="n">
-        <v>790</v>
-      </c>
-      <c r="J7" t="inlineStr">
+        <v>995</v>
+      </c>
+      <c r="H7" t="inlineStr">
         <is>
           <t>3/3</t>
         </is>
       </c>
-      <c r="K7" t="n">
+      <c r="I7" t="n">
         <v>200</v>
       </c>
     </row>
@@ -1557,23 +1573,20 @@
         </is>
       </c>
       <c r="E8" t="n">
-        <v>693</v>
+        <v>636</v>
       </c>
       <c r="F8" t="n">
-        <v>594</v>
+        <v>661</v>
       </c>
       <c r="G8" t="n">
-        <v>744</v>
-      </c>
-      <c r="H8" t="n">
-        <v>813</v>
-      </c>
-      <c r="J8" t="inlineStr">
+        <v>787</v>
+      </c>
+      <c r="H8" t="inlineStr">
         <is>
           <t>3/3</t>
         </is>
       </c>
-      <c r="K8" t="n">
+      <c r="I8" t="n">
         <v>200</v>
       </c>
     </row>
@@ -1597,23 +1610,20 @@
         </is>
       </c>
       <c r="E9" t="n">
-        <v>690</v>
+        <v>616</v>
       </c>
       <c r="F9" t="n">
-        <v>655</v>
+        <v>643</v>
       </c>
       <c r="G9" t="n">
-        <v>722</v>
-      </c>
-      <c r="H9" t="n">
-        <v>874</v>
-      </c>
-      <c r="J9" t="inlineStr">
+        <v>788</v>
+      </c>
+      <c r="H9" t="inlineStr">
         <is>
           <t>3/3</t>
         </is>
       </c>
-      <c r="K9" t="n">
+      <c r="I9" t="n">
         <v>200</v>
       </c>
     </row>
@@ -1637,23 +1647,20 @@
         </is>
       </c>
       <c r="E10" t="n">
-        <v>400</v>
+        <v>620</v>
       </c>
       <c r="F10" t="n">
-        <v>390</v>
+        <v>624</v>
       </c>
       <c r="G10" t="n">
-        <v>423</v>
-      </c>
-      <c r="H10" t="n">
-        <v>966</v>
-      </c>
-      <c r="J10" t="inlineStr">
+        <v>1177</v>
+      </c>
+      <c r="H10" t="inlineStr">
         <is>
           <t>3/3</t>
         </is>
       </c>
-      <c r="K10" t="n">
+      <c r="I10" t="n">
         <v>200</v>
       </c>
     </row>
@@ -1677,23 +1684,20 @@
         </is>
       </c>
       <c r="E11" t="n">
-        <v>466</v>
+        <v>630</v>
       </c>
       <c r="F11" t="n">
-        <v>392</v>
+        <v>634</v>
       </c>
       <c r="G11" t="n">
-        <v>470</v>
-      </c>
-      <c r="H11" t="n">
-        <v>1042</v>
-      </c>
-      <c r="J11" t="inlineStr">
+        <v>1259</v>
+      </c>
+      <c r="H11" t="inlineStr">
         <is>
           <t>3/3</t>
         </is>
       </c>
-      <c r="K11" t="n">
+      <c r="I11" t="n">
         <v>200</v>
       </c>
     </row>
@@ -1717,23 +1721,20 @@
         </is>
       </c>
       <c r="E12" t="n">
-        <v>420</v>
+        <v>650</v>
       </c>
       <c r="F12" t="n">
-        <v>412</v>
+        <v>654</v>
       </c>
       <c r="G12" t="n">
-        <v>457</v>
-      </c>
-      <c r="H12" t="n">
-        <v>980</v>
-      </c>
-      <c r="J12" t="inlineStr">
+        <v>1193</v>
+      </c>
+      <c r="H12" t="inlineStr">
         <is>
           <t>3/3</t>
         </is>
       </c>
-      <c r="K12" t="n">
+      <c r="I12" t="n">
         <v>200</v>
       </c>
     </row>
@@ -1757,35 +1758,32 @@
         </is>
       </c>
       <c r="E13" t="n">
-        <v>455</v>
+        <v>621</v>
       </c>
       <c r="F13" t="n">
-        <v>429</v>
+        <v>624</v>
       </c>
       <c r="G13" t="n">
-        <v>456</v>
-      </c>
-      <c r="H13" t="n">
-        <v>1119</v>
-      </c>
-      <c r="J13" t="inlineStr">
+        <v>1310</v>
+      </c>
+      <c r="H13" t="inlineStr">
         <is>
           <t>3/3</t>
         </is>
       </c>
-      <c r="K13" t="n">
+      <c r="I13" t="n">
         <v>200</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Atlas</t>
+          <t>Deepgram</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>ja</t>
+          <t>en</t>
         </is>
       </c>
       <c r="C14" t="n">
@@ -1793,42 +1791,36 @@
       </c>
       <c r="D14" s="3" t="inlineStr">
         <is>
-          <t>お電話ありがとうございます。本日はどのようなご用件でしょうか。</t>
+          <t>Thank you for calling Manulife Finance, how may I help you today?</t>
         </is>
       </c>
       <c r="E14" t="n">
-        <v>919</v>
+        <v>1007</v>
       </c>
       <c r="F14" t="n">
-        <v>902</v>
+        <v>1267</v>
       </c>
       <c r="G14" t="n">
-        <v>1036</v>
-      </c>
-      <c r="H14" t="n">
-        <v>2133</v>
+        <v>1508</v>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>3/3</t>
+        </is>
       </c>
       <c r="I14" t="n">
-        <v>322</v>
-      </c>
-      <c r="J14" t="inlineStr">
-        <is>
-          <t>3/3</t>
-        </is>
-      </c>
-      <c r="K14" t="n">
         <v>200</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Atlas</t>
+          <t>Deepgram</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>ja</t>
+          <t>en</t>
         </is>
       </c>
       <c r="C15" t="n">
@@ -1836,42 +1828,36 @@
       </c>
       <c r="D15" s="3" t="inlineStr">
         <is>
-          <t>医療保険と生命保険について詳しく教えてください。</t>
+          <t>I would like to transfer five thousand dollars to my savings account.</t>
         </is>
       </c>
       <c r="E15" t="n">
-        <v>946</v>
+        <v>1171</v>
       </c>
       <c r="F15" t="n">
-        <v>880</v>
+        <v>1396</v>
       </c>
       <c r="G15" t="n">
-        <v>956</v>
-      </c>
-      <c r="H15" t="n">
-        <v>2135</v>
+        <v>1623</v>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>3/3</t>
+        </is>
       </c>
       <c r="I15" t="n">
-        <v>333</v>
-      </c>
-      <c r="J15" t="inlineStr">
-        <is>
-          <t>3/3</t>
-        </is>
-      </c>
-      <c r="K15" t="n">
         <v>200</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Atlas</t>
+          <t>Deepgram</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>ja</t>
+          <t>en</t>
         </is>
       </c>
       <c r="C16" t="n">
@@ -1879,42 +1865,36 @@
       </c>
       <c r="D16" s="3" t="inlineStr">
         <is>
-          <t>来月の保険料の支払い方法を変更したいのですが。</t>
+          <t>Can you tell me about term life insurance and medical coverage?</t>
         </is>
       </c>
       <c r="E16" t="n">
-        <v>989</v>
+        <v>1095</v>
       </c>
       <c r="F16" t="n">
-        <v>965</v>
+        <v>1314</v>
       </c>
       <c r="G16" t="n">
-        <v>1432</v>
-      </c>
-      <c r="H16" t="n">
-        <v>2401</v>
+        <v>1541</v>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>3/3</t>
+        </is>
       </c>
       <c r="I16" t="n">
-        <v>335</v>
-      </c>
-      <c r="J16" t="inlineStr">
-        <is>
-          <t>3/3</t>
-        </is>
-      </c>
-      <c r="K16" t="n">
         <v>200</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Atlas</t>
+          <t>Deepgram</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>ja</t>
+          <t>en</t>
         </is>
       </c>
       <c r="C17" t="n">
@@ -1922,37 +1902,31 @@
       </c>
       <c r="D17" s="3" t="inlineStr">
         <is>
-          <t>担当者に相談の予約をお願いできますか。</t>
+          <t>My policy number is one two three four five six, and my name is Jayant.</t>
         </is>
       </c>
       <c r="E17" t="n">
-        <v>960</v>
+        <v>963</v>
       </c>
       <c r="F17" t="n">
-        <v>923</v>
+        <v>1212</v>
       </c>
       <c r="G17" t="n">
-        <v>1130</v>
-      </c>
-      <c r="H17" t="n">
-        <v>2034</v>
+        <v>1470</v>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>3/3</t>
+        </is>
       </c>
       <c r="I17" t="n">
-        <v>525</v>
-      </c>
-      <c r="J17" t="inlineStr">
-        <is>
-          <t>3/3</t>
-        </is>
-      </c>
-      <c r="K17" t="n">
         <v>200</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>ElevenLabs</t>
+          <t>Atlas</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -1969,30 +1943,27 @@
         </is>
       </c>
       <c r="E18" t="n">
-        <v>690</v>
+        <v>1116</v>
       </c>
       <c r="F18" t="n">
-        <v>644</v>
+        <v>1225</v>
       </c>
       <c r="G18" t="n">
-        <v>719</v>
-      </c>
-      <c r="H18" t="n">
-        <v>782</v>
-      </c>
-      <c r="J18" t="inlineStr">
+        <v>2507</v>
+      </c>
+      <c r="H18" t="inlineStr">
         <is>
           <t>3/3</t>
         </is>
       </c>
-      <c r="K18" t="n">
+      <c r="I18" t="n">
         <v>200</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>ElevenLabs</t>
+          <t>Atlas</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -2009,30 +1980,27 @@
         </is>
       </c>
       <c r="E19" t="n">
-        <v>667</v>
+        <v>1032</v>
       </c>
       <c r="F19" t="n">
-        <v>646</v>
+        <v>1139</v>
       </c>
       <c r="G19" t="n">
-        <v>716</v>
-      </c>
-      <c r="H19" t="n">
-        <v>763</v>
-      </c>
-      <c r="J19" t="inlineStr">
+        <v>2373</v>
+      </c>
+      <c r="H19" t="inlineStr">
         <is>
           <t>3/3</t>
         </is>
       </c>
-      <c r="K19" t="n">
+      <c r="I19" t="n">
         <v>200</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>ElevenLabs</t>
+          <t>Atlas</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -2049,30 +2017,27 @@
         </is>
       </c>
       <c r="E20" t="n">
-        <v>647</v>
+        <v>981</v>
       </c>
       <c r="F20" t="n">
-        <v>618</v>
+        <v>1088</v>
       </c>
       <c r="G20" t="n">
-        <v>752</v>
-      </c>
-      <c r="H20" t="n">
-        <v>732</v>
-      </c>
-      <c r="J20" t="inlineStr">
+        <v>2481</v>
+      </c>
+      <c r="H20" t="inlineStr">
         <is>
           <t>3/3</t>
         </is>
       </c>
-      <c r="K20" t="n">
+      <c r="I20" t="n">
         <v>200</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>ElevenLabs</t>
+          <t>Atlas</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -2089,30 +2054,27 @@
         </is>
       </c>
       <c r="E21" t="n">
-        <v>702</v>
+        <v>981</v>
       </c>
       <c r="F21" t="n">
-        <v>670</v>
+        <v>1096</v>
       </c>
       <c r="G21" t="n">
-        <v>745</v>
-      </c>
-      <c r="H21" t="n">
-        <v>818</v>
-      </c>
-      <c r="J21" t="inlineStr">
+        <v>2139</v>
+      </c>
+      <c r="H21" t="inlineStr">
         <is>
           <t>3/3</t>
         </is>
       </c>
-      <c r="K21" t="n">
+      <c r="I21" t="n">
         <v>200</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Cartesia</t>
+          <t>ElevenLabs</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -2129,30 +2091,27 @@
         </is>
       </c>
       <c r="E22" t="n">
-        <v>414</v>
+        <v>802</v>
       </c>
       <c r="F22" t="n">
-        <v>382</v>
+        <v>835</v>
       </c>
       <c r="G22" t="n">
-        <v>449</v>
-      </c>
-      <c r="H22" t="n">
-        <v>1208</v>
-      </c>
-      <c r="J22" t="inlineStr">
+        <v>915</v>
+      </c>
+      <c r="H22" t="inlineStr">
         <is>
           <t>3/3</t>
         </is>
       </c>
-      <c r="K22" t="n">
+      <c r="I22" t="n">
         <v>200</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Cartesia</t>
+          <t>ElevenLabs</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -2169,30 +2128,27 @@
         </is>
       </c>
       <c r="E23" t="n">
-        <v>427</v>
+        <v>830</v>
       </c>
       <c r="F23" t="n">
-        <v>387</v>
+        <v>860</v>
       </c>
       <c r="G23" t="n">
-        <v>555</v>
-      </c>
-      <c r="H23" t="n">
-        <v>1110</v>
-      </c>
-      <c r="J23" t="inlineStr">
+        <v>943</v>
+      </c>
+      <c r="H23" t="inlineStr">
         <is>
           <t>3/3</t>
         </is>
       </c>
-      <c r="K23" t="n">
+      <c r="I23" t="n">
         <v>200</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Cartesia</t>
+          <t>ElevenLabs</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -2209,30 +2165,27 @@
         </is>
       </c>
       <c r="E24" t="n">
-        <v>399</v>
+        <v>818</v>
       </c>
       <c r="F24" t="n">
-        <v>397</v>
+        <v>853</v>
       </c>
       <c r="G24" t="n">
-        <v>428</v>
-      </c>
-      <c r="H24" t="n">
-        <v>1062</v>
-      </c>
-      <c r="J24" t="inlineStr">
+        <v>938</v>
+      </c>
+      <c r="H24" t="inlineStr">
         <is>
           <t>3/3</t>
         </is>
       </c>
-      <c r="K24" t="n">
+      <c r="I24" t="n">
         <v>200</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Cartesia</t>
+          <t>ElevenLabs</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -2249,24 +2202,289 @@
         </is>
       </c>
       <c r="E25" t="n">
-        <v>427</v>
+        <v>868</v>
       </c>
       <c r="F25" t="n">
-        <v>395</v>
+        <v>906</v>
       </c>
       <c r="G25" t="n">
-        <v>460</v>
-      </c>
-      <c r="H25" t="n">
-        <v>938</v>
-      </c>
-      <c r="J25" t="inlineStr">
+        <v>970</v>
+      </c>
+      <c r="H25" t="inlineStr">
         <is>
           <t>3/3</t>
         </is>
       </c>
-      <c r="K25" t="n">
+      <c r="I25" t="n">
         <v>200</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>Cartesia</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="C26" t="n">
+        <v>0</v>
+      </c>
+      <c r="D26" s="3" t="inlineStr">
+        <is>
+          <t>お電話ありがとうございます。本日はどのようなご用件でしょうか。</t>
+        </is>
+      </c>
+      <c r="E26" t="n">
+        <v>700</v>
+      </c>
+      <c r="F26" t="n">
+        <v>704</v>
+      </c>
+      <c r="G26" t="n">
+        <v>1559</v>
+      </c>
+      <c r="H26" t="inlineStr">
+        <is>
+          <t>3/3</t>
+        </is>
+      </c>
+      <c r="I26" t="n">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>Cartesia</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="C27" t="n">
+        <v>1</v>
+      </c>
+      <c r="D27" s="3" t="inlineStr">
+        <is>
+          <t>医療保険と生命保険について詳しく教えてください。</t>
+        </is>
+      </c>
+      <c r="E27" t="n">
+        <v>692</v>
+      </c>
+      <c r="F27" t="n">
+        <v>695</v>
+      </c>
+      <c r="G27" t="n">
+        <v>1277</v>
+      </c>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>3/3</t>
+        </is>
+      </c>
+      <c r="I27" t="n">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>Cartesia</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="C28" t="n">
+        <v>2</v>
+      </c>
+      <c r="D28" s="3" t="inlineStr">
+        <is>
+          <t>来月の保険料の支払い方法を変更したいのですが。</t>
+        </is>
+      </c>
+      <c r="E28" t="n">
+        <v>661</v>
+      </c>
+      <c r="F28" t="n">
+        <v>665</v>
+      </c>
+      <c r="G28" t="n">
+        <v>1271</v>
+      </c>
+      <c r="H28" t="inlineStr">
+        <is>
+          <t>3/3</t>
+        </is>
+      </c>
+      <c r="I28" t="n">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>Cartesia</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="C29" t="n">
+        <v>3</v>
+      </c>
+      <c r="D29" s="3" t="inlineStr">
+        <is>
+          <t>担当者に相談の予約をお願いできますか。</t>
+        </is>
+      </c>
+      <c r="E29" t="n">
+        <v>432</v>
+      </c>
+      <c r="F29" t="n">
+        <v>435</v>
+      </c>
+      <c r="G29" t="n">
+        <v>883</v>
+      </c>
+      <c r="H29" t="inlineStr">
+        <is>
+          <t>3/3</t>
+        </is>
+      </c>
+      <c r="I29" t="n">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>Deepgram</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="C30" t="n">
+        <v>0</v>
+      </c>
+      <c r="D30" s="3" t="inlineStr">
+        <is>
+          <t>お電話ありがとうございます。本日はどのようなご用件でしょうか。</t>
+        </is>
+      </c>
+      <c r="H30" t="inlineStr">
+        <is>
+          <t>0/3</t>
+        </is>
+      </c>
+      <c r="I30" t="inlineStr">
+        <is>
+          <t>N/A (English only)</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>Deepgram</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="C31" t="n">
+        <v>1</v>
+      </c>
+      <c r="D31" s="3" t="inlineStr">
+        <is>
+          <t>医療保険と生命保険について詳しく教えてください。</t>
+        </is>
+      </c>
+      <c r="H31" t="inlineStr">
+        <is>
+          <t>0/3</t>
+        </is>
+      </c>
+      <c r="I31" t="inlineStr">
+        <is>
+          <t>N/A (English only)</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>Deepgram</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="C32" t="n">
+        <v>2</v>
+      </c>
+      <c r="D32" s="3" t="inlineStr">
+        <is>
+          <t>来月の保険料の支払い方法を変更したいのですが。</t>
+        </is>
+      </c>
+      <c r="H32" t="inlineStr">
+        <is>
+          <t>0/3</t>
+        </is>
+      </c>
+      <c r="I32" t="inlineStr">
+        <is>
+          <t>N/A (English only)</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>Deepgram</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="C33" t="n">
+        <v>3</v>
+      </c>
+      <c r="D33" s="3" t="inlineStr">
+        <is>
+          <t>担当者に相談の予約をお願いできますか。</t>
+        </is>
+      </c>
+      <c r="H33" t="inlineStr">
+        <is>
+          <t>0/3</t>
+        </is>
+      </c>
+      <c r="I33" t="inlineStr">
+        <is>
+          <t>N/A (English only)</t>
+        </is>
       </c>
     </row>
   </sheetData>
@@ -2280,7 +2498,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K25"/>
+  <dimension ref="A1:I33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2290,10 +2508,8 @@
     <col width="45" customWidth="1" min="5" max="5"/>
     <col width="8" customWidth="1" min="6" max="6"/>
     <col width="12" customWidth="1" min="7" max="7"/>
-    <col width="10" customWidth="1" min="8" max="8"/>
-    <col width="12" customWidth="1" min="9" max="9"/>
-    <col width="20" customWidth="1" min="10" max="10"/>
-    <col width="10" customWidth="1" min="11" max="11"/>
+    <col width="12" customWidth="1" min="8" max="8"/>
+    <col width="30" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2314,7 +2530,7 @@
       </c>
       <c r="D1" s="5" t="inlineStr">
         <is>
-          <t>Reference (correct text)</t>
+          <t>Reference (correct)</t>
         </is>
       </c>
       <c r="E1" s="5" t="inlineStr">
@@ -2334,22 +2550,12 @@
       </c>
       <c r="H1" s="5" t="inlineStr">
         <is>
-          <t>Error rate</t>
+          <t>Latency (ms)</t>
         </is>
       </c>
       <c r="I1" s="5" t="inlineStr">
         <is>
-          <t>Latency (ms)</t>
-        </is>
-      </c>
-      <c r="J1" s="5" t="inlineStr">
-        <is>
           <t>Mode</t>
-        </is>
-      </c>
-      <c r="K1" s="5" t="inlineStr">
-        <is>
-          <t>Status</t>
         </is>
       </c>
     </row>
@@ -2386,24 +2592,18 @@
         <v>100</v>
       </c>
       <c r="H2" t="n">
-        <v>0</v>
-      </c>
-      <c r="I2" t="n">
-        <v>2377</v>
-      </c>
-      <c r="J2" t="inlineStr">
-        <is>
-          <t>sync</t>
-        </is>
-      </c>
-      <c r="K2" t="n">
-        <v>200</v>
+        <v>378</v>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>streaming (time to first word)</t>
+        </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Deepgram</t>
+          <t>ElevenLabs</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -2419,38 +2619,28 @@
           <t>Thank you for calling Manulife Finance, how may I help you today?</t>
         </is>
       </c>
-      <c r="E3" s="3" t="inlineStr">
-        <is>
-          <t>Thank you for calling Manulife Finance. How may I help you today?</t>
-        </is>
-      </c>
+      <c r="E3" s="3" t="inlineStr"/>
       <c r="F3" t="inlineStr">
         <is>
           <t>WER</t>
         </is>
       </c>
       <c r="G3" t="n">
-        <v>100</v>
+        <v>0</v>
       </c>
       <c r="H3" t="n">
-        <v>0</v>
-      </c>
-      <c r="I3" t="n">
-        <v>1309</v>
-      </c>
-      <c r="J3" t="inlineStr">
+        <v>1238</v>
+      </c>
+      <c r="I3" t="inlineStr">
         <is>
           <t>sync</t>
         </is>
-      </c>
-      <c r="K3" t="n">
-        <v>200</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>AssemblyAI</t>
+          <t>Deepgram</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -2480,26 +2670,18 @@
         <v>100</v>
       </c>
       <c r="H4" t="n">
-        <v>0</v>
-      </c>
-      <c r="I4" t="n">
-        <v>5991</v>
-      </c>
-      <c r="J4" t="inlineStr">
-        <is>
-          <t>batch (upload+poll)</t>
-        </is>
-      </c>
-      <c r="K4" t="inlineStr">
-        <is>
-          <t>completed</t>
+        <v>730</v>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>streaming (time to first word)</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Atlas</t>
+          <t>AssemblyAI</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -2508,16 +2690,16 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D5" s="3" t="inlineStr">
         <is>
-          <t>I would like to transfer five thousand dollars to my savings account.</t>
+          <t>Thank you for calling Manulife Finance, how may I help you today?</t>
         </is>
       </c>
       <c r="E5" s="3" t="inlineStr">
         <is>
-          <t>I would like to transfer $5,000 to my savings account.</t>
+          <t>Thank you for calling Manulife Finance. How may I help you today?</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
@@ -2526,27 +2708,21 @@
         </is>
       </c>
       <c r="G5" t="n">
-        <v>75</v>
+        <v>100</v>
       </c>
       <c r="H5" t="n">
-        <v>0.25</v>
-      </c>
-      <c r="I5" t="n">
-        <v>2494</v>
-      </c>
-      <c r="J5" t="inlineStr">
-        <is>
-          <t>sync</t>
-        </is>
-      </c>
-      <c r="K5" t="n">
-        <v>200</v>
+        <v>6034</v>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>batch (upload+poll)</t>
+        </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Deepgram</t>
+          <t>Atlas</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -2576,24 +2752,18 @@
         <v>75</v>
       </c>
       <c r="H6" t="n">
-        <v>0.25</v>
-      </c>
-      <c r="I6" t="n">
-        <v>1383</v>
-      </c>
-      <c r="J6" t="inlineStr">
-        <is>
-          <t>sync</t>
-        </is>
-      </c>
-      <c r="K6" t="n">
-        <v>200</v>
+        <v>348</v>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>streaming (time to first word)</t>
+        </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>AssemblyAI</t>
+          <t>ElevenLabs</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -2609,40 +2779,28 @@
           <t>I would like to transfer five thousand dollars to my savings account.</t>
         </is>
       </c>
-      <c r="E7" s="3" t="inlineStr">
-        <is>
-          <t>I would like to transfer $5,000 to my savings account.</t>
-        </is>
-      </c>
+      <c r="E7" s="3" t="inlineStr"/>
       <c r="F7" t="inlineStr">
         <is>
           <t>WER</t>
         </is>
       </c>
       <c r="G7" t="n">
-        <v>75</v>
+        <v>0</v>
       </c>
       <c r="H7" t="n">
-        <v>0.25</v>
-      </c>
-      <c r="I7" t="n">
-        <v>5273</v>
-      </c>
-      <c r="J7" t="inlineStr">
-        <is>
-          <t>batch (upload+poll)</t>
-        </is>
-      </c>
-      <c r="K7" t="inlineStr">
-        <is>
-          <t>completed</t>
+        <v>1240</v>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>sync</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Atlas</t>
+          <t>Deepgram</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -2651,16 +2809,16 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D8" s="3" t="inlineStr">
         <is>
-          <t>Can you tell me about term life insurance and medical coverage?</t>
+          <t>I would like to transfer five thousand dollars to my savings account.</t>
         </is>
       </c>
       <c r="E8" s="3" t="inlineStr">
         <is>
-          <t>Can you tell me about term life insurance and medical coverage?</t>
+          <t>I would like to transfer five thousand dollars to my savings account.</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
@@ -2672,24 +2830,18 @@
         <v>100</v>
       </c>
       <c r="H8" t="n">
-        <v>0</v>
-      </c>
-      <c r="I8" t="n">
-        <v>2284</v>
-      </c>
-      <c r="J8" t="inlineStr">
-        <is>
-          <t>sync</t>
-        </is>
-      </c>
-      <c r="K8" t="n">
-        <v>200</v>
+        <v>735</v>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>streaming (time to first word)</t>
+        </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Deepgram</t>
+          <t>AssemblyAI</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
@@ -2698,16 +2850,16 @@
         </is>
       </c>
       <c r="C9" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D9" s="3" t="inlineStr">
         <is>
-          <t>Can you tell me about term life insurance and medical coverage?</t>
+          <t>I would like to transfer five thousand dollars to my savings account.</t>
         </is>
       </c>
       <c r="E9" s="3" t="inlineStr">
         <is>
-          <t>Can you tell me about term life insurance and medical coverage?</t>
+          <t>I would like to transfer $5,000 to my savings account.</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
@@ -2716,27 +2868,21 @@
         </is>
       </c>
       <c r="G9" t="n">
-        <v>100</v>
+        <v>75</v>
       </c>
       <c r="H9" t="n">
-        <v>0</v>
-      </c>
-      <c r="I9" t="n">
-        <v>1328</v>
-      </c>
-      <c r="J9" t="inlineStr">
-        <is>
-          <t>sync</t>
-        </is>
-      </c>
-      <c r="K9" t="n">
-        <v>200</v>
+        <v>5781</v>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>batch (upload+poll)</t>
+        </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>AssemblyAI</t>
+          <t>Atlas</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -2766,26 +2912,18 @@
         <v>100</v>
       </c>
       <c r="H10" t="n">
-        <v>0</v>
-      </c>
-      <c r="I10" t="n">
-        <v>6622</v>
-      </c>
-      <c r="J10" t="inlineStr">
-        <is>
-          <t>batch (upload+poll)</t>
-        </is>
-      </c>
-      <c r="K10" t="inlineStr">
-        <is>
-          <t>completed</t>
+        <v>387</v>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>streaming (time to first word)</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Atlas</t>
+          <t>ElevenLabs</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -2794,39 +2932,29 @@
         </is>
       </c>
       <c r="C11" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D11" s="3" t="inlineStr">
         <is>
-          <t>My policy number is one two three four five six, and my name is Jayant.</t>
-        </is>
-      </c>
-      <c r="E11" s="3" t="inlineStr">
-        <is>
-          <t>My policy number is 123-456, and my name is Jayant.</t>
-        </is>
-      </c>
+          <t>Can you tell me about term life insurance and medical coverage?</t>
+        </is>
+      </c>
+      <c r="E11" s="3" t="inlineStr"/>
       <c r="F11" t="inlineStr">
         <is>
           <t>WER</t>
         </is>
       </c>
       <c r="G11" t="n">
-        <v>60</v>
+        <v>0</v>
       </c>
       <c r="H11" t="n">
-        <v>0.4</v>
-      </c>
-      <c r="I11" t="n">
-        <v>3270</v>
-      </c>
-      <c r="J11" t="inlineStr">
+        <v>1039</v>
+      </c>
+      <c r="I11" t="inlineStr">
         <is>
           <t>sync</t>
         </is>
-      </c>
-      <c r="K11" t="n">
-        <v>200</v>
       </c>
     </row>
     <row r="12">
@@ -2841,16 +2969,16 @@
         </is>
       </c>
       <c r="C12" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D12" s="3" t="inlineStr">
         <is>
-          <t>My policy number is one two three four five six, and my name is Jayant.</t>
+          <t>Can you tell me about term life insurance and medical coverage?</t>
         </is>
       </c>
       <c r="E12" s="3" t="inlineStr">
         <is>
-          <t>My policy number is 123456, and my name is Jayant.</t>
+          <t>Can you tell me about term life insurance and medical coverage?</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
@@ -2859,21 +2987,15 @@
         </is>
       </c>
       <c r="G12" t="n">
-        <v>60</v>
+        <v>100</v>
       </c>
       <c r="H12" t="n">
-        <v>0.4</v>
-      </c>
-      <c r="I12" t="n">
-        <v>1543</v>
-      </c>
-      <c r="J12" t="inlineStr">
-        <is>
-          <t>sync</t>
-        </is>
-      </c>
-      <c r="K12" t="n">
-        <v>200</v>
+        <v>728</v>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>streaming (time to first word)</t>
+        </is>
       </c>
     </row>
     <row r="13">
@@ -2888,16 +3010,16 @@
         </is>
       </c>
       <c r="C13" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D13" s="3" t="inlineStr">
         <is>
-          <t>My policy number is one two three four five six, and my name is Jayant.</t>
+          <t>Can you tell me about term life insurance and medical coverage?</t>
         </is>
       </c>
       <c r="E13" s="3" t="inlineStr">
         <is>
-          <t>My policy number is 123456, and my name is Jayant.</t>
+          <t>Can you tell me about term life insurance and medical coverage?</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
@@ -2906,22 +3028,14 @@
         </is>
       </c>
       <c r="G13" t="n">
-        <v>60</v>
+        <v>100</v>
       </c>
       <c r="H13" t="n">
-        <v>0.4</v>
-      </c>
-      <c r="I13" t="n">
-        <v>5173</v>
-      </c>
-      <c r="J13" t="inlineStr">
+        <v>5740</v>
+      </c>
+      <c r="I13" t="inlineStr">
         <is>
           <t>batch (upload+poll)</t>
-        </is>
-      </c>
-      <c r="K13" t="inlineStr">
-        <is>
-          <t>completed</t>
         </is>
       </c>
     </row>
@@ -2933,192 +3047,162 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>ja</t>
+          <t>en</t>
         </is>
       </c>
       <c r="C14" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="D14" s="3" t="inlineStr">
         <is>
-          <t>お電話ありがとうございます。本日はどのようなご用件でしょうか。</t>
+          <t>My policy number is one two three four five six, and my name is Jayant.</t>
         </is>
       </c>
       <c r="E14" s="3" t="inlineStr">
         <is>
-          <t>お電話ありがとうございます。本日はどのようなご用件でしょうか。</t>
+          <t>My policy number is 123456, and my name is Jayant.</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>CER</t>
+          <t>WER</t>
         </is>
       </c>
       <c r="G14" t="n">
-        <v>100</v>
+        <v>60</v>
       </c>
       <c r="H14" t="n">
-        <v>0</v>
-      </c>
-      <c r="I14" t="n">
-        <v>2704</v>
-      </c>
-      <c r="J14" t="inlineStr">
-        <is>
-          <t>sync</t>
-        </is>
-      </c>
-      <c r="K14" t="n">
-        <v>200</v>
+        <v>384</v>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>streaming (time to first word)</t>
+        </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Deepgram</t>
+          <t>ElevenLabs</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>ja</t>
+          <t>en</t>
         </is>
       </c>
       <c r="C15" t="n">
+        <v>3</v>
+      </c>
+      <c r="D15" s="3" t="inlineStr">
+        <is>
+          <t>My policy number is one two three four five six, and my name is Jayant.</t>
+        </is>
+      </c>
+      <c r="E15" s="3" t="inlineStr"/>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>WER</t>
+        </is>
+      </c>
+      <c r="G15" t="n">
         <v>0</v>
       </c>
-      <c r="D15" s="3" t="inlineStr">
-        <is>
-          <t>お電話ありがとうございます。本日はどのようなご用件でしょうか。</t>
-        </is>
-      </c>
-      <c r="E15" s="3" t="inlineStr">
-        <is>
-          <t>お電話、ありがとうございます。本日はどのようなご用件でしょうか。</t>
-        </is>
-      </c>
-      <c r="F15" t="inlineStr">
-        <is>
-          <t>CER</t>
-        </is>
-      </c>
-      <c r="G15" t="n">
-        <v>100</v>
-      </c>
       <c r="H15" t="n">
-        <v>0</v>
-      </c>
-      <c r="I15" t="n">
-        <v>1997</v>
-      </c>
-      <c r="J15" t="inlineStr">
+        <v>1059</v>
+      </c>
+      <c r="I15" t="inlineStr">
         <is>
           <t>sync</t>
         </is>
-      </c>
-      <c r="K15" t="n">
-        <v>200</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>AssemblyAI</t>
+          <t>Deepgram</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>ja</t>
+          <t>en</t>
         </is>
       </c>
       <c r="C16" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="D16" s="3" t="inlineStr">
         <is>
-          <t>お電話ありがとうございます。本日はどのようなご用件でしょうか。</t>
+          <t>My policy number is one two three four five six, and my name is Jayant.</t>
         </is>
       </c>
       <c r="E16" s="3" t="inlineStr">
         <is>
-          <t>お電話ありがとうございます。本日はどのようなご要件でしょうか。</t>
+          <t>My policy number is one two three four five six and my name is Jayant.</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>CER</t>
+          <t>WER</t>
         </is>
       </c>
       <c r="G16" t="n">
-        <v>96.59999999999999</v>
+        <v>100</v>
       </c>
       <c r="H16" t="n">
-        <v>0.034</v>
-      </c>
-      <c r="I16" t="n">
-        <v>5122</v>
-      </c>
-      <c r="J16" t="inlineStr">
-        <is>
-          <t>batch (upload+poll)</t>
-        </is>
-      </c>
-      <c r="K16" t="inlineStr">
-        <is>
-          <t>completed</t>
+        <v>736</v>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>streaming (time to first word)</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Atlas</t>
+          <t>AssemblyAI</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>ja</t>
+          <t>en</t>
         </is>
       </c>
       <c r="C17" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D17" s="3" t="inlineStr">
         <is>
-          <t>医療保険と生命保険について詳しく教えてください。</t>
+          <t>My policy number is one two three four five six, and my name is Jayant.</t>
         </is>
       </c>
       <c r="E17" s="3" t="inlineStr">
         <is>
-          <t>医療保険と生命保険について、詳しく教えてください。</t>
+          <t>My policy number is 123456, and my name is Jayant.</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>CER</t>
+          <t>WER</t>
         </is>
       </c>
       <c r="G17" t="n">
-        <v>100</v>
+        <v>60</v>
       </c>
       <c r="H17" t="n">
-        <v>0</v>
-      </c>
-      <c r="I17" t="n">
-        <v>2639</v>
-      </c>
-      <c r="J17" t="inlineStr">
-        <is>
-          <t>sync</t>
-        </is>
-      </c>
-      <c r="K17" t="n">
-        <v>200</v>
+        <v>6005</v>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>batch (upload+poll)</t>
+        </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Deepgram</t>
+          <t>Atlas</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -3127,16 +3211,16 @@
         </is>
       </c>
       <c r="C18" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D18" s="3" t="inlineStr">
         <is>
-          <t>医療保険と生命保険について詳しく教えてください。</t>
+          <t>お電話ありがとうございます。本日はどのようなご用件でしょうか。</t>
         </is>
       </c>
       <c r="E18" s="3" t="inlineStr">
         <is>
-          <t>医療保険と生命保険について詳しく教えてください</t>
+          <t>お電話ありがとうございます。本日はどのようなご用件でしょうか。</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
@@ -3148,24 +3232,18 @@
         <v>100</v>
       </c>
       <c r="H18" t="n">
-        <v>0</v>
-      </c>
-      <c r="I18" t="n">
-        <v>1578</v>
-      </c>
-      <c r="J18" t="inlineStr">
-        <is>
-          <t>sync</t>
-        </is>
-      </c>
-      <c r="K18" t="n">
-        <v>200</v>
+        <v>444</v>
+      </c>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>streaming (time to first word)</t>
+        </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>AssemblyAI</t>
+          <t>ElevenLabs</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -3174,47 +3252,35 @@
         </is>
       </c>
       <c r="C19" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D19" s="3" t="inlineStr">
         <is>
-          <t>医療保険と生命保険について詳しく教えてください。</t>
-        </is>
-      </c>
-      <c r="E19" s="3" t="inlineStr">
-        <is>
-          <t>医療保険と生命保険について詳しく知ってください。</t>
-        </is>
-      </c>
+          <t>お電話ありがとうございます。本日はどのようなご用件でしょうか。</t>
+        </is>
+      </c>
+      <c r="E19" s="3" t="inlineStr"/>
       <c r="F19" t="inlineStr">
         <is>
           <t>CER</t>
         </is>
       </c>
       <c r="G19" t="n">
-        <v>91.3</v>
+        <v>0</v>
       </c>
       <c r="H19" t="n">
-        <v>0.08699999999999999</v>
-      </c>
-      <c r="I19" t="n">
-        <v>5312</v>
-      </c>
-      <c r="J19" t="inlineStr">
-        <is>
-          <t>batch (upload+poll)</t>
-        </is>
-      </c>
-      <c r="K19" t="inlineStr">
-        <is>
-          <t>completed</t>
+        <v>1170</v>
+      </c>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>sync</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Atlas</t>
+          <t>Deepgram</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -3223,16 +3289,16 @@
         </is>
       </c>
       <c r="C20" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="D20" s="3" t="inlineStr">
         <is>
-          <t>来月の保険料の支払い方法を変更したいのですが。</t>
+          <t>お電話ありがとうございます。本日はどのようなご用件でしょうか。</t>
         </is>
       </c>
       <c r="E20" s="3" t="inlineStr">
         <is>
-          <t>来月の保険料の支払い方法を変更したいのですが、—</t>
+          <t>電話ありがとうございます。 本日はどのようなご用件でしょうか。</t>
         </is>
       </c>
       <c r="F20" t="inlineStr">
@@ -3241,27 +3307,21 @@
         </is>
       </c>
       <c r="G20" t="n">
-        <v>95.5</v>
+        <v>96.59999999999999</v>
       </c>
       <c r="H20" t="n">
-        <v>0.045</v>
-      </c>
-      <c r="I20" t="n">
-        <v>2583</v>
-      </c>
-      <c r="J20" t="inlineStr">
-        <is>
-          <t>sync</t>
-        </is>
-      </c>
-      <c r="K20" t="n">
-        <v>200</v>
+        <v>776</v>
+      </c>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>streaming (time to first word)</t>
+        </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Deepgram</t>
+          <t>AssemblyAI</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -3270,16 +3330,16 @@
         </is>
       </c>
       <c r="C21" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="D21" s="3" t="inlineStr">
         <is>
-          <t>来月の保険料の支払い方法を変更したいのですが。</t>
+          <t>お電話ありがとうございます。本日はどのようなご用件でしょうか。</t>
         </is>
       </c>
       <c r="E21" s="3" t="inlineStr">
         <is>
-          <t>来月の保険料の支払い方法を変更したいのですが</t>
+          <t>お電話ありがとうございます。本日はどのようなご要件でしょうか。</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
@@ -3288,27 +3348,21 @@
         </is>
       </c>
       <c r="G21" t="n">
-        <v>100</v>
+        <v>96.59999999999999</v>
       </c>
       <c r="H21" t="n">
-        <v>0</v>
-      </c>
-      <c r="I21" t="n">
-        <v>3040</v>
-      </c>
-      <c r="J21" t="inlineStr">
-        <is>
-          <t>sync</t>
-        </is>
-      </c>
-      <c r="K21" t="n">
-        <v>200</v>
+        <v>5708</v>
+      </c>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>batch (upload+poll)</t>
+        </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>AssemblyAI</t>
+          <t>Atlas</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -3317,16 +3371,16 @@
         </is>
       </c>
       <c r="C22" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D22" s="3" t="inlineStr">
         <is>
-          <t>来月の保険料の支払い方法を変更したいのですが。</t>
+          <t>医療保険と生命保険について詳しく教えてください。</t>
         </is>
       </c>
       <c r="E22" s="3" t="inlineStr">
         <is>
-          <t>来月の保険料の支払い方法を変更したいのですが。</t>
+          <t>医療保険と生命保険について詳しく教えてください。</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
@@ -3338,26 +3392,18 @@
         <v>100</v>
       </c>
       <c r="H22" t="n">
-        <v>0</v>
-      </c>
-      <c r="I22" t="n">
-        <v>5249</v>
-      </c>
-      <c r="J22" t="inlineStr">
-        <is>
-          <t>batch (upload+poll)</t>
-        </is>
-      </c>
-      <c r="K22" t="inlineStr">
-        <is>
-          <t>completed</t>
+        <v>443</v>
+      </c>
+      <c r="I22" t="inlineStr">
+        <is>
+          <t>streaming (time to first word)</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Atlas</t>
+          <t>ElevenLabs</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -3366,39 +3412,29 @@
         </is>
       </c>
       <c r="C23" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D23" s="3" t="inlineStr">
         <is>
-          <t>担当者に相談の予約をお願いできますか。</t>
-        </is>
-      </c>
-      <c r="E23" s="3" t="inlineStr">
-        <is>
-          <t>担当者に相談の予約をお願いできますか。</t>
-        </is>
-      </c>
+          <t>医療保険と生命保険について詳しく教えてください。</t>
+        </is>
+      </c>
+      <c r="E23" s="3" t="inlineStr"/>
       <c r="F23" t="inlineStr">
         <is>
           <t>CER</t>
         </is>
       </c>
       <c r="G23" t="n">
-        <v>100</v>
+        <v>0</v>
       </c>
       <c r="H23" t="n">
-        <v>0</v>
-      </c>
-      <c r="I23" t="n">
-        <v>2198</v>
-      </c>
-      <c r="J23" t="inlineStr">
+        <v>1376</v>
+      </c>
+      <c r="I23" t="inlineStr">
         <is>
           <t>sync</t>
         </is>
-      </c>
-      <c r="K23" t="n">
-        <v>200</v>
       </c>
     </row>
     <row r="24">
@@ -3413,16 +3449,16 @@
         </is>
       </c>
       <c r="C24" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D24" s="3" t="inlineStr">
         <is>
-          <t>担当者に相談の予約をお願いできますか。</t>
+          <t>医療保険と生命保険について詳しく教えてください。</t>
         </is>
       </c>
       <c r="E24" s="3" t="inlineStr">
         <is>
-          <t>担当者に相談の予約をお願いできますか</t>
+          <t>医療保険と生命保険について詳しく教えてください。</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
@@ -3434,18 +3470,12 @@
         <v>100</v>
       </c>
       <c r="H24" t="n">
-        <v>0</v>
-      </c>
-      <c r="I24" t="n">
-        <v>1541</v>
-      </c>
-      <c r="J24" t="inlineStr">
-        <is>
-          <t>sync</t>
-        </is>
-      </c>
-      <c r="K24" t="n">
-        <v>200</v>
+        <v>773</v>
+      </c>
+      <c r="I24" t="inlineStr">
+        <is>
+          <t>streaming (time to first word)</t>
+        </is>
       </c>
     </row>
     <row r="25">
@@ -3460,16 +3490,16 @@
         </is>
       </c>
       <c r="C25" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D25" s="3" t="inlineStr">
         <is>
-          <t>担当者に相談の予約をお願いできますか。</t>
+          <t>医療保険と生命保険について詳しく教えてください。</t>
         </is>
       </c>
       <c r="E25" s="3" t="inlineStr">
         <is>
-          <t>担当者に相談の予約をお願いできますか?</t>
+          <t>医療保険と生命保険について詳しく教えてください。</t>
         </is>
       </c>
       <c r="F25" t="inlineStr">
@@ -3481,19 +3511,331 @@
         <v>100</v>
       </c>
       <c r="H25" t="n">
+        <v>6757</v>
+      </c>
+      <c r="I25" t="inlineStr">
+        <is>
+          <t>batch (upload+poll)</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>Atlas</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="C26" t="n">
+        <v>2</v>
+      </c>
+      <c r="D26" s="3" t="inlineStr">
+        <is>
+          <t>来月の保険料の支払い方法を変更したいのですが。</t>
+        </is>
+      </c>
+      <c r="E26" s="3" t="inlineStr">
+        <is>
+          <t>来月の保険料の支払い方法を変更したいのですが。</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>CER</t>
+        </is>
+      </c>
+      <c r="G26" t="n">
+        <v>100</v>
+      </c>
+      <c r="H26" t="n">
+        <v>454</v>
+      </c>
+      <c r="I26" t="inlineStr">
+        <is>
+          <t>streaming (time to first word)</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>ElevenLabs</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="C27" t="n">
+        <v>2</v>
+      </c>
+      <c r="D27" s="3" t="inlineStr">
+        <is>
+          <t>来月の保険料の支払い方法を変更したいのですが。</t>
+        </is>
+      </c>
+      <c r="E27" s="3" t="inlineStr"/>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>CER</t>
+        </is>
+      </c>
+      <c r="G27" t="n">
         <v>0</v>
       </c>
-      <c r="I25" t="n">
-        <v>5006</v>
-      </c>
-      <c r="J25" t="inlineStr">
+      <c r="H27" t="n">
+        <v>2437</v>
+      </c>
+      <c r="I27" t="inlineStr">
+        <is>
+          <t>sync</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>Deepgram</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="C28" t="n">
+        <v>2</v>
+      </c>
+      <c r="D28" s="3" t="inlineStr">
+        <is>
+          <t>来月の保険料の支払い方法を変更したいのですが。</t>
+        </is>
+      </c>
+      <c r="E28" s="3" t="inlineStr">
+        <is>
+          <t>来月の保険料の支払い方法を変更したいのですが</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>CER</t>
+        </is>
+      </c>
+      <c r="G28" t="n">
+        <v>100</v>
+      </c>
+      <c r="H28" t="n">
+        <v>785</v>
+      </c>
+      <c r="I28" t="inlineStr">
+        <is>
+          <t>streaming (time to first word)</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>AssemblyAI</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="C29" t="n">
+        <v>2</v>
+      </c>
+      <c r="D29" s="3" t="inlineStr">
+        <is>
+          <t>来月の保険料の支払い方法を変更したいのですが。</t>
+        </is>
+      </c>
+      <c r="E29" s="3" t="inlineStr">
+        <is>
+          <t>来月の保険料の支払い方法を変更したいのですが。</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>CER</t>
+        </is>
+      </c>
+      <c r="G29" t="n">
+        <v>100</v>
+      </c>
+      <c r="H29" t="n">
+        <v>6261</v>
+      </c>
+      <c r="I29" t="inlineStr">
         <is>
           <t>batch (upload+poll)</t>
         </is>
       </c>
-      <c r="K25" t="inlineStr">
-        <is>
-          <t>completed</t>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>Atlas</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="C30" t="n">
+        <v>3</v>
+      </c>
+      <c r="D30" s="3" t="inlineStr">
+        <is>
+          <t>担当者に相談の予約をお願いできますか。</t>
+        </is>
+      </c>
+      <c r="E30" s="3" t="inlineStr">
+        <is>
+          <t>担当者に相談の予約をお願いできますか。</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>CER</t>
+        </is>
+      </c>
+      <c r="G30" t="n">
+        <v>100</v>
+      </c>
+      <c r="H30" t="n">
+        <v>463</v>
+      </c>
+      <c r="I30" t="inlineStr">
+        <is>
+          <t>streaming (time to first word)</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>ElevenLabs</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="C31" t="n">
+        <v>3</v>
+      </c>
+      <c r="D31" s="3" t="inlineStr">
+        <is>
+          <t>担当者に相談の予約をお願いできますか。</t>
+        </is>
+      </c>
+      <c r="E31" s="3" t="inlineStr"/>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>CER</t>
+        </is>
+      </c>
+      <c r="G31" t="n">
+        <v>0</v>
+      </c>
+      <c r="H31" t="n">
+        <v>1218</v>
+      </c>
+      <c r="I31" t="inlineStr">
+        <is>
+          <t>sync</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>Deepgram</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="C32" t="n">
+        <v>3</v>
+      </c>
+      <c r="D32" s="3" t="inlineStr">
+        <is>
+          <t>担当者に相談の予約をお願いできますか。</t>
+        </is>
+      </c>
+      <c r="E32" s="3" t="inlineStr">
+        <is>
+          <t>担当者に相談の予約をお願いできますか。</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>CER</t>
+        </is>
+      </c>
+      <c r="G32" t="n">
+        <v>100</v>
+      </c>
+      <c r="H32" t="n">
+        <v>757</v>
+      </c>
+      <c r="I32" t="inlineStr">
+        <is>
+          <t>streaming (time to first word)</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>AssemblyAI</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>ja</t>
+        </is>
+      </c>
+      <c r="C33" t="n">
+        <v>3</v>
+      </c>
+      <c r="D33" s="3" t="inlineStr">
+        <is>
+          <t>担当者に相談の予約をお願いできますか。</t>
+        </is>
+      </c>
+      <c r="E33" s="3" t="inlineStr">
+        <is>
+          <t>担当者に相談の予約をお願いできますか?</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>CER</t>
+        </is>
+      </c>
+      <c r="G33" t="n">
+        <v>100</v>
+      </c>
+      <c r="H33" t="n">
+        <v>6310</v>
+      </c>
+      <c r="I33" t="inlineStr">
+        <is>
+          <t>batch (upload+poll)</t>
         </is>
       </c>
     </row>

</xml_diff>